<commit_message>
cmb-s4 has been cancelled; add results for simons observatory
</commit_message>
<xml_diff>
--- a/code/cmb/all.xlsx
+++ b/code/cmb/all.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -487,34 +487,34 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>185128827.2032204</v>
+        <v>214783404.6453064</v>
       </c>
       <c r="C2" t="n">
-        <v>-692898147.965669</v>
+        <v>-754176437.6587168</v>
       </c>
       <c r="D2" t="n">
-        <v>137105704.1822474</v>
+        <v>165064299.6061957</v>
       </c>
       <c r="E2" t="n">
-        <v>-4740935.5909728</v>
+        <v>-4990171.094117044</v>
       </c>
       <c r="F2" t="n">
-        <v>-57824336.49902042</v>
+        <v>-67932432.35814896</v>
       </c>
       <c r="G2" t="n">
-        <v>-12447147.39915775</v>
+        <v>-14775494.22321544</v>
       </c>
       <c r="H2" t="n">
-        <v>-6589565.032637624</v>
+        <v>-7638291.459668837</v>
       </c>
       <c r="I2" t="n">
-        <v>44850335.90973126</v>
+        <v>52851790.52852885</v>
       </c>
       <c r="J2" t="n">
-        <v>1850758.676345401</v>
+        <v>1526208.647273082</v>
       </c>
       <c r="K2" t="n">
-        <v>113623.7762489748</v>
+        <v>-43858.24048372477</v>
       </c>
     </row>
     <row r="3">
@@ -524,34 +524,34 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-692898147.965669</v>
+        <v>-754176437.6587168</v>
       </c>
       <c r="C3" t="n">
-        <v>3023402063.7132</v>
+        <v>3045160151.929213</v>
       </c>
       <c r="D3" t="n">
-        <v>-458354152.9478175</v>
+        <v>-532229663.5078512</v>
       </c>
       <c r="E3" t="n">
-        <v>32060982.8601459</v>
+        <v>32201582.09118408</v>
       </c>
       <c r="F3" t="n">
-        <v>222609446.857868</v>
+        <v>243037661.7363127</v>
       </c>
       <c r="G3" t="n">
-        <v>47145032.98248264</v>
+        <v>51765994.45441859</v>
       </c>
       <c r="H3" t="n">
-        <v>23282304.91692092</v>
+        <v>25676869.25873105</v>
       </c>
       <c r="I3" t="n">
-        <v>-171421945.9644465</v>
+        <v>-187602318.4623074</v>
       </c>
       <c r="J3" t="n">
-        <v>-7598366.941132234</v>
+        <v>-7272187.80199012</v>
       </c>
       <c r="K3" t="n">
-        <v>-577001.0976232829</v>
+        <v>-347201.4778237099</v>
       </c>
     </row>
     <row r="4">
@@ -561,34 +561,34 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>137105704.1822474</v>
+        <v>165064299.6061957</v>
       </c>
       <c r="C4" t="n">
-        <v>-458354152.9478175</v>
+        <v>-532229663.5078512</v>
       </c>
       <c r="D4" t="n">
-        <v>112570195.9145628</v>
+        <v>137153141.0927557</v>
       </c>
       <c r="E4" t="n">
-        <v>-1894717.528196103</v>
+        <v>-2256316.008823832</v>
       </c>
       <c r="F4" t="n">
-        <v>-38173852.29402938</v>
+        <v>-47122260.1775704</v>
       </c>
       <c r="G4" t="n">
-        <v>-7840065.595027551</v>
+        <v>-9843027.753381327</v>
       </c>
       <c r="H4" t="n">
-        <v>-5484485.3914593</v>
+        <v>-6503293.58918516</v>
       </c>
       <c r="I4" t="n">
-        <v>29626603.15036413</v>
+        <v>36696859.37530451</v>
       </c>
       <c r="J4" t="n">
-        <v>3552607.696506803</v>
+        <v>3577964.593454808</v>
       </c>
       <c r="K4" t="n">
-        <v>706066.2423816043</v>
+        <v>651471.937061148</v>
       </c>
     </row>
     <row r="5">
@@ -598,34 +598,34 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-4740935.5909728</v>
+        <v>-4990171.094117044</v>
       </c>
       <c r="C5" t="n">
-        <v>32060982.8601459</v>
+        <v>32201582.09118408</v>
       </c>
       <c r="D5" t="n">
-        <v>-1894717.528196103</v>
+        <v>-2256316.008823832</v>
       </c>
       <c r="E5" t="n">
-        <v>1046894.876764914</v>
+        <v>1126557.128860747</v>
       </c>
       <c r="F5" t="n">
-        <v>1665062.528972976</v>
+        <v>1775017.118698751</v>
       </c>
       <c r="G5" t="n">
-        <v>314995.9056964207</v>
+        <v>331757.6426421268</v>
       </c>
       <c r="H5" t="n">
-        <v>112570.0547995077</v>
+        <v>119163.4128697279</v>
       </c>
       <c r="I5" t="n">
-        <v>-1284038.782650934</v>
+        <v>-1355803.827674127</v>
       </c>
       <c r="J5" t="n">
-        <v>-136068.6251404728</v>
+        <v>-147876.040647799</v>
       </c>
       <c r="K5" t="n">
-        <v>-25864.90841879048</v>
+        <v>-28437.05677293328</v>
       </c>
     </row>
     <row r="6">
@@ -635,34 +635,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-57824336.49902042</v>
+        <v>-67932432.35814896</v>
       </c>
       <c r="C6" t="n">
-        <v>222609446.857868</v>
+        <v>243037661.7363127</v>
       </c>
       <c r="D6" t="n">
-        <v>-38173852.29402937</v>
+        <v>-47122260.1775704</v>
       </c>
       <c r="E6" t="n">
-        <v>1665062.528972976</v>
+        <v>1775017.11869875</v>
       </c>
       <c r="F6" t="n">
-        <v>22361670.04211807</v>
+        <v>26524674.36798792</v>
       </c>
       <c r="G6" t="n">
-        <v>5252308.014423977</v>
+        <v>6277010.36769974</v>
       </c>
       <c r="H6" t="n">
-        <v>1591678.691991868</v>
+        <v>1876784.017298848</v>
       </c>
       <c r="I6" t="n">
-        <v>-17311887.25329487</v>
+        <v>-20607860.58270219</v>
       </c>
       <c r="J6" t="n">
-        <v>1719658.543695215</v>
+        <v>2218885.873207679</v>
       </c>
       <c r="K6" t="n">
-        <v>615137.948390104</v>
+        <v>778936.3366697851</v>
       </c>
     </row>
     <row r="7">
@@ -672,34 +672,34 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-12447147.39915775</v>
+        <v>-14775494.22321544</v>
       </c>
       <c r="C7" t="n">
-        <v>47145032.98248264</v>
+        <v>51765994.45441859</v>
       </c>
       <c r="D7" t="n">
-        <v>-7840065.595027551</v>
+        <v>-9843027.753381327</v>
       </c>
       <c r="E7" t="n">
-        <v>314995.9056964208</v>
+        <v>331757.6426421268</v>
       </c>
       <c r="F7" t="n">
-        <v>5252308.014423977</v>
+        <v>6277010.36769974</v>
       </c>
       <c r="G7" t="n">
-        <v>1282974.971498364</v>
+        <v>1541394.214566836</v>
       </c>
       <c r="H7" t="n">
-        <v>294682.0272687076</v>
+        <v>354051.3710280803</v>
       </c>
       <c r="I7" t="n">
-        <v>-4090355.805696196</v>
+        <v>-4902867.615305995</v>
       </c>
       <c r="J7" t="n">
-        <v>636982.0494556346</v>
+        <v>790860.1855230279</v>
       </c>
       <c r="K7" t="n">
-        <v>207844.8676078545</v>
+        <v>256559.8393645194</v>
       </c>
     </row>
     <row r="8">
@@ -709,34 +709,34 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-6589565.032637624</v>
+        <v>-7638291.459668837</v>
       </c>
       <c r="C8" t="n">
-        <v>23282304.91692092</v>
+        <v>25676869.25873105</v>
       </c>
       <c r="D8" t="n">
-        <v>-5484485.3914593</v>
+        <v>-6503293.58918516</v>
       </c>
       <c r="E8" t="n">
-        <v>112570.0547995077</v>
+        <v>119163.4128697279</v>
       </c>
       <c r="F8" t="n">
-        <v>1591678.691991868</v>
+        <v>1876784.017298847</v>
       </c>
       <c r="G8" t="n">
-        <v>294682.0272687076</v>
+        <v>354051.3710280803</v>
       </c>
       <c r="H8" t="n">
-        <v>288494.3636698526</v>
+        <v>332463.0425229847</v>
       </c>
       <c r="I8" t="n">
-        <v>-1230549.691288918</v>
+        <v>-1457024.979927192</v>
       </c>
       <c r="J8" t="n">
-        <v>-314171.6836654741</v>
+        <v>-341228.1776014238</v>
       </c>
       <c r="K8" t="n">
-        <v>-74443.62774460834</v>
+        <v>-79794.08612457081</v>
       </c>
     </row>
     <row r="9">
@@ -746,34 +746,34 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>44850335.90973125</v>
+        <v>52851790.52852885</v>
       </c>
       <c r="C9" t="n">
-        <v>-171421945.9644465</v>
+        <v>-187602318.4623074</v>
       </c>
       <c r="D9" t="n">
-        <v>29626603.15036413</v>
+        <v>36696859.37530451</v>
       </c>
       <c r="E9" t="n">
-        <v>-1284038.782650934</v>
+        <v>-1355803.827674127</v>
       </c>
       <c r="F9" t="n">
-        <v>-17311887.25329487</v>
+        <v>-20607860.58270219</v>
       </c>
       <c r="G9" t="n">
-        <v>-4090355.805696196</v>
+        <v>-4902867.615305995</v>
       </c>
       <c r="H9" t="n">
-        <v>-1230549.691288918</v>
+        <v>-1457024.979927192</v>
       </c>
       <c r="I9" t="n">
-        <v>13743610.01478225</v>
+        <v>16353728.71888681</v>
       </c>
       <c r="J9" t="n">
-        <v>-1374591.952840707</v>
+        <v>-1773296.995894149</v>
       </c>
       <c r="K9" t="n">
-        <v>-488745.1873570743</v>
+        <v>-619360.5477270398</v>
       </c>
     </row>
     <row r="10">
@@ -783,34 +783,34 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1850758.676345401</v>
+        <v>1526208.647273082</v>
       </c>
       <c r="C10" t="n">
-        <v>-7598366.941132233</v>
+        <v>-7272187.801990118</v>
       </c>
       <c r="D10" t="n">
-        <v>3552607.696506803</v>
+        <v>3577964.593454808</v>
       </c>
       <c r="E10" t="n">
-        <v>-136068.6251404728</v>
+        <v>-147876.040647799</v>
       </c>
       <c r="F10" t="n">
-        <v>1719658.543695215</v>
+        <v>2218885.873207679</v>
       </c>
       <c r="G10" t="n">
-        <v>636982.0494556346</v>
+        <v>790860.1855230279</v>
       </c>
       <c r="H10" t="n">
-        <v>-314171.6836654741</v>
+        <v>-341228.1776014238</v>
       </c>
       <c r="I10" t="n">
-        <v>-1374591.952840707</v>
+        <v>-1773296.995894149</v>
       </c>
       <c r="J10" t="n">
-        <v>1329265.687606041</v>
+        <v>1552170.519826235</v>
       </c>
       <c r="K10" t="n">
-        <v>371850.3956049974</v>
+        <v>435641.8322264933</v>
       </c>
     </row>
     <row r="11">
@@ -820,34 +820,34 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>113623.7762489748</v>
+        <v>-43858.24048372474</v>
       </c>
       <c r="C11" t="n">
-        <v>-577001.0976232829</v>
+        <v>-347201.4778237098</v>
       </c>
       <c r="D11" t="n">
-        <v>706066.2423816042</v>
+        <v>651471.937061148</v>
       </c>
       <c r="E11" t="n">
-        <v>-25864.90841879048</v>
+        <v>-28437.05677293327</v>
       </c>
       <c r="F11" t="n">
-        <v>615137.948390104</v>
+        <v>778936.3366697851</v>
       </c>
       <c r="G11" t="n">
-        <v>207844.8676078545</v>
+        <v>256559.8393645195</v>
       </c>
       <c r="H11" t="n">
-        <v>-74443.62774460834</v>
+        <v>-79794.08612457081</v>
       </c>
       <c r="I11" t="n">
-        <v>-488745.1873570743</v>
+        <v>-619360.5477270397</v>
       </c>
       <c r="J11" t="n">
-        <v>371850.3956049974</v>
+        <v>435641.8322264933</v>
       </c>
       <c r="K11" t="n">
-        <v>104924.4609376661</v>
+        <v>123324.1641093451</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
only use so lat mf band
</commit_message>
<xml_diff>
--- a/code/cmb/all.xlsx
+++ b/code/cmb/all.xlsx
@@ -487,34 +487,34 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>214783404.6453064</v>
+        <v>211315691.5881169</v>
       </c>
       <c r="C2" t="n">
-        <v>-754176437.6587168</v>
+        <v>-739146092.5912594</v>
       </c>
       <c r="D2" t="n">
-        <v>165064299.6061957</v>
+        <v>162654350.079329</v>
       </c>
       <c r="E2" t="n">
-        <v>-4990171.094117044</v>
+        <v>-4834303.960672051</v>
       </c>
       <c r="F2" t="n">
-        <v>-67932432.35814896</v>
+        <v>-66934310.34504158</v>
       </c>
       <c r="G2" t="n">
-        <v>-14775494.22321544</v>
+        <v>-14576886.65685084</v>
       </c>
       <c r="H2" t="n">
-        <v>-7638291.459668837</v>
+        <v>-7508163.466622662</v>
       </c>
       <c r="I2" t="n">
-        <v>52851790.52852885</v>
+        <v>52089225.71584815</v>
       </c>
       <c r="J2" t="n">
-        <v>1526208.647273082</v>
+        <v>1425683.867425521</v>
       </c>
       <c r="K2" t="n">
-        <v>-43858.24048372477</v>
+        <v>-64524.04032347223</v>
       </c>
     </row>
     <row r="3">
@@ -524,34 +524,34 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-754176437.6587168</v>
+        <v>-739146092.5912594</v>
       </c>
       <c r="C3" t="n">
-        <v>3045160151.929213</v>
+        <v>2972794610.213633</v>
       </c>
       <c r="D3" t="n">
-        <v>-532229663.5078512</v>
+        <v>-523089194.3522037</v>
       </c>
       <c r="E3" t="n">
-        <v>32201582.09118408</v>
+        <v>31369632.26980191</v>
       </c>
       <c r="F3" t="n">
-        <v>243037661.7363127</v>
+        <v>238318257.2192546</v>
       </c>
       <c r="G3" t="n">
-        <v>51765994.45441859</v>
+        <v>50789722.75702452</v>
       </c>
       <c r="H3" t="n">
-        <v>25676869.25873105</v>
+        <v>25169054.58710053</v>
       </c>
       <c r="I3" t="n">
-        <v>-187602318.4623074</v>
+        <v>-183997434.1953858</v>
       </c>
       <c r="J3" t="n">
-        <v>-7272187.80199012</v>
+        <v>-7019564.406528383</v>
       </c>
       <c r="K3" t="n">
-        <v>-347201.4778237099</v>
+        <v>-309843.7663926973</v>
       </c>
     </row>
     <row r="4">
@@ -561,34 +561,34 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>165064299.6061957</v>
+        <v>162654350.079329</v>
       </c>
       <c r="C4" t="n">
-        <v>-532229663.5078512</v>
+        <v>-523089194.3522037</v>
       </c>
       <c r="D4" t="n">
-        <v>137153141.0927557</v>
+        <v>135185251.4216629</v>
       </c>
       <c r="E4" t="n">
-        <v>-2256316.008823832</v>
+        <v>-2179861.466628375</v>
       </c>
       <c r="F4" t="n">
-        <v>-47122260.1775704</v>
+        <v>-46557934.49603374</v>
       </c>
       <c r="G4" t="n">
-        <v>-9843027.753381327</v>
+        <v>-9745313.718872994</v>
       </c>
       <c r="H4" t="n">
-        <v>-6503293.58918516</v>
+        <v>-6396045.248333052</v>
       </c>
       <c r="I4" t="n">
-        <v>36696859.37530451</v>
+        <v>36268492.47512119</v>
       </c>
       <c r="J4" t="n">
-        <v>3577964.593454808</v>
+        <v>3441884.727025041</v>
       </c>
       <c r="K4" t="n">
-        <v>651471.937061148</v>
+        <v>618290.9471532184</v>
       </c>
     </row>
     <row r="5">
@@ -598,34 +598,34 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-4990171.094117044</v>
+        <v>-4834303.960672051</v>
       </c>
       <c r="C5" t="n">
-        <v>32201582.09118408</v>
+        <v>31369632.26980191</v>
       </c>
       <c r="D5" t="n">
-        <v>-2256316.008823832</v>
+        <v>-2179861.466628375</v>
       </c>
       <c r="E5" t="n">
-        <v>1126557.128860747</v>
+        <v>1112812.271201333</v>
       </c>
       <c r="F5" t="n">
-        <v>1775017.118698751</v>
+        <v>1717749.246002197</v>
       </c>
       <c r="G5" t="n">
-        <v>331757.6426421268</v>
+        <v>318956.1159544929</v>
       </c>
       <c r="H5" t="n">
-        <v>119163.4128697279</v>
+        <v>115237.483665062</v>
       </c>
       <c r="I5" t="n">
-        <v>-1355803.827674127</v>
+        <v>-1311011.717318675</v>
       </c>
       <c r="J5" t="n">
-        <v>-147876.040647799</v>
+        <v>-149502.7130061111</v>
       </c>
       <c r="K5" t="n">
-        <v>-28437.05677293328</v>
+        <v>-29267.89960267367</v>
       </c>
     </row>
     <row r="6">
@@ -635,34 +635,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-67932432.35814896</v>
+        <v>-66934310.34504158</v>
       </c>
       <c r="C6" t="n">
-        <v>243037661.7363127</v>
+        <v>238318257.2192546</v>
       </c>
       <c r="D6" t="n">
-        <v>-47122260.1775704</v>
+        <v>-46557934.49603374</v>
       </c>
       <c r="E6" t="n">
-        <v>1775017.11869875</v>
+        <v>1717749.246002197</v>
       </c>
       <c r="F6" t="n">
-        <v>26524674.36798792</v>
+        <v>26146055.98059578</v>
       </c>
       <c r="G6" t="n">
-        <v>6277010.36769974</v>
+        <v>6191751.56921301</v>
       </c>
       <c r="H6" t="n">
-        <v>1876784.017298848</v>
+        <v>1849825.984405096</v>
       </c>
       <c r="I6" t="n">
-        <v>-20607860.58270219</v>
+        <v>-20319854.2164714</v>
       </c>
       <c r="J6" t="n">
-        <v>2218885.873207679</v>
+        <v>2201249.162468201</v>
       </c>
       <c r="K6" t="n">
-        <v>778936.3366697851</v>
+        <v>771688.9570959039</v>
       </c>
     </row>
     <row r="7">
@@ -672,34 +672,34 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-14775494.22321544</v>
+        <v>-14576886.65685084</v>
       </c>
       <c r="C7" t="n">
-        <v>51765994.45441859</v>
+        <v>50789722.75702452</v>
       </c>
       <c r="D7" t="n">
-        <v>-9843027.753381327</v>
+        <v>-9745313.718872994</v>
       </c>
       <c r="E7" t="n">
-        <v>331757.6426421268</v>
+        <v>318956.1159544929</v>
       </c>
       <c r="F7" t="n">
-        <v>6277010.36769974</v>
+        <v>6191751.56921301</v>
       </c>
       <c r="G7" t="n">
-        <v>1541394.214566836</v>
+        <v>1521176.985645031</v>
       </c>
       <c r="H7" t="n">
-        <v>354051.3710280803</v>
+        <v>349893.4863207093</v>
       </c>
       <c r="I7" t="n">
-        <v>-4902867.615305995</v>
+        <v>-4837492.546285028</v>
       </c>
       <c r="J7" t="n">
-        <v>790860.1855230279</v>
+        <v>781882.2425580018</v>
       </c>
       <c r="K7" t="n">
-        <v>256559.8393645194</v>
+        <v>253566.5287063388</v>
       </c>
     </row>
     <row r="8">
@@ -709,34 +709,34 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-7638291.459668837</v>
+        <v>-7508163.466622662</v>
       </c>
       <c r="C8" t="n">
-        <v>25676869.25873105</v>
+        <v>25169054.58710053</v>
       </c>
       <c r="D8" t="n">
-        <v>-6503293.58918516</v>
+        <v>-6396045.248333052</v>
       </c>
       <c r="E8" t="n">
-        <v>119163.4128697279</v>
+        <v>115237.483665062</v>
       </c>
       <c r="F8" t="n">
-        <v>1876784.017298847</v>
+        <v>1849825.984405096</v>
       </c>
       <c r="G8" t="n">
-        <v>354051.3710280803</v>
+        <v>349893.4863207093</v>
       </c>
       <c r="H8" t="n">
-        <v>332463.0425229847</v>
+        <v>326299.9297667388</v>
       </c>
       <c r="I8" t="n">
-        <v>-1457024.979927192</v>
+        <v>-1436582.711952711</v>
       </c>
       <c r="J8" t="n">
-        <v>-341228.1776014238</v>
+        <v>-331994.7524050627</v>
       </c>
       <c r="K8" t="n">
-        <v>-79794.08612457081</v>
+        <v>-77468.97128414043</v>
       </c>
     </row>
     <row r="9">
@@ -746,34 +746,34 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>52851790.52852885</v>
+        <v>52089225.71584815</v>
       </c>
       <c r="C9" t="n">
-        <v>-187602318.4623074</v>
+        <v>-183997434.1953858</v>
       </c>
       <c r="D9" t="n">
-        <v>36696859.37530451</v>
+        <v>36268492.47512119</v>
       </c>
       <c r="E9" t="n">
-        <v>-1355803.827674127</v>
+        <v>-1311011.717318675</v>
       </c>
       <c r="F9" t="n">
-        <v>-20607860.58270219</v>
+        <v>-20319854.2164714</v>
       </c>
       <c r="G9" t="n">
-        <v>-4902867.615305995</v>
+        <v>-4837492.546285028</v>
       </c>
       <c r="H9" t="n">
-        <v>-1457024.979927192</v>
+        <v>-1436582.711952711</v>
       </c>
       <c r="I9" t="n">
-        <v>16353728.71888681</v>
+        <v>16132444.53118232</v>
       </c>
       <c r="J9" t="n">
-        <v>-1773296.995894149</v>
+        <v>-1759260.680454546</v>
       </c>
       <c r="K9" t="n">
-        <v>-619360.5477270398</v>
+        <v>-613654.6790766082</v>
       </c>
     </row>
     <row r="10">
@@ -783,34 +783,34 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1526208.647273082</v>
+        <v>1425683.867425521</v>
       </c>
       <c r="C10" t="n">
-        <v>-7272187.801990118</v>
+        <v>-7019564.406528383</v>
       </c>
       <c r="D10" t="n">
-        <v>3577964.593454808</v>
+        <v>3441884.727025041</v>
       </c>
       <c r="E10" t="n">
-        <v>-147876.040647799</v>
+        <v>-149502.7130061111</v>
       </c>
       <c r="F10" t="n">
-        <v>2218885.873207679</v>
+        <v>2201249.162468201</v>
       </c>
       <c r="G10" t="n">
-        <v>790860.1855230279</v>
+        <v>781882.2425580018</v>
       </c>
       <c r="H10" t="n">
-        <v>-341228.1776014238</v>
+        <v>-331994.7524050627</v>
       </c>
       <c r="I10" t="n">
-        <v>-1773296.995894149</v>
+        <v>-1759260.680454546</v>
       </c>
       <c r="J10" t="n">
-        <v>1552170.519826235</v>
+        <v>1524647.947919311</v>
       </c>
       <c r="K10" t="n">
-        <v>435641.8322264933</v>
+        <v>428067.7644063422</v>
       </c>
     </row>
     <row r="11">
@@ -820,34 +820,34 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-43858.24048372474</v>
+        <v>-64524.04032347215</v>
       </c>
       <c r="C11" t="n">
-        <v>-347201.4778237098</v>
+        <v>-309843.7663926971</v>
       </c>
       <c r="D11" t="n">
-        <v>651471.937061148</v>
+        <v>618290.9471532184</v>
       </c>
       <c r="E11" t="n">
-        <v>-28437.05677293327</v>
+        <v>-29267.89960267366</v>
       </c>
       <c r="F11" t="n">
-        <v>778936.3366697851</v>
+        <v>771688.9570959039</v>
       </c>
       <c r="G11" t="n">
-        <v>256559.8393645195</v>
+        <v>253566.5287063388</v>
       </c>
       <c r="H11" t="n">
-        <v>-79794.08612457081</v>
+        <v>-77468.97128414043</v>
       </c>
       <c r="I11" t="n">
-        <v>-619360.5477270397</v>
+        <v>-613654.6790766082</v>
       </c>
       <c r="J11" t="n">
-        <v>435641.8322264933</v>
+        <v>428067.7644063422</v>
       </c>
       <c r="K11" t="n">
-        <v>123324.1641093451</v>
+        <v>121223.9358656424</v>
       </c>
     </row>
   </sheetData>

</xml_diff>